<commit_message>
Sync PRD, tech spec, and mockup: remove rollback, fix ObjectId, exact decimal precision, add clear history
</commit_message>
<xml_diff>
--- a/data/LAE-44136/CTR 0422.xlsx
+++ b/data/LAE-44136/CTR 0422.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nakisainc-my.sharepoint.com/personal/cfulger_nakisa_com/Documents/Documents/Abbott/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{061E60F3-CD66-4189-A6F1-ED5824894615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{061E60F3-CD66-4189-A6F1-ED5824894615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{198F02D7-35B4-4830-AA1C-13637C454931}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{4B450442-8F7A-4F2B-B61B-922CCE2E4D9A}"/>
   </bookViews>
@@ -18,11 +18,11 @@
     <sheet name="Remeasurement" sheetId="1" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CTR '!$A$27:$BP$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CTR '!$A$27:$BP$42</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="20" r:id="rId4"/>
+    <pivotCache cacheId="25" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="189">
   <si>
     <t>Contract Currency</t>
   </si>
@@ -587,6 +587,30 @@
   </si>
   <si>
     <t>P&amp;L</t>
+  </si>
+  <si>
+    <t>CTR "R"</t>
+  </si>
+  <si>
+    <t>CTR "AX"</t>
+  </si>
+  <si>
+    <t>CTR "AY"</t>
+  </si>
+  <si>
+    <t>Mapping</t>
+  </si>
+  <si>
+    <t>CTR "BF" only symbol</t>
+  </si>
+  <si>
+    <t>sum of all entries</t>
+  </si>
+  <si>
+    <t>CAD</t>
+  </si>
+  <si>
+    <t>CTR "BH" symbol only</t>
   </si>
 </sst>
 </file>
@@ -847,7 +871,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -971,21 +995,39 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="9" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="49" fontId="7" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="10" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2302,7 +2344,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9DF64DB8-525B-4071-A21F-1CC2319F23F6}" name="PivotTable3" cacheId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9DF64DB8-525B-4071-A21F-1CC2319F23F6}" name="PivotTable3" cacheId="25" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:D12" firstHeaderRow="0" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="68">
     <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
@@ -2784,6 +2826,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9401912A-04DC-40F6-9E6F-836BB5DB28BF}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:BP42"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2859,7 +2902,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>41</v>
       </c>
       <c r="B1" s="46"/>
@@ -2869,7 +2912,7 @@
       <c r="F1" s="46"/>
     </row>
     <row r="2" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="49" t="s">
         <v>42</v>
       </c>
       <c r="B2" s="46"/>
@@ -2879,15 +2922,15 @@
       <c r="F2" s="46"/>
     </row>
     <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.35">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="50" t="s">
         <v>43</v>
       </c>
       <c r="B3" s="46"/>
-      <c r="C3" s="48" t="s">
+      <c r="C3" s="50" t="s">
         <v>44</v>
       </c>
       <c r="D3" s="46"/>
-      <c r="E3" s="48" t="s">
+      <c r="E3" s="50" t="s">
         <v>45</v>
       </c>
       <c r="F3" s="46"/>
@@ -2933,10 +2976,10 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="49" t="s">
+      <c r="A6" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="47" t="s">
         <v>57</v>
       </c>
       <c r="C6" s="28" t="s">
@@ -3250,7 +3293,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="28" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="29" t="s">
         <v>138</v>
       </c>
@@ -3394,7 +3437,7 @@
       <c r="BO28" s="35"/>
       <c r="BP28" s="34"/>
     </row>
-    <row r="29" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="29" t="s">
         <v>138</v>
       </c>
@@ -3538,7 +3581,7 @@
       <c r="BO29" s="35"/>
       <c r="BP29" s="34"/>
     </row>
-    <row r="30" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="29" t="s">
         <v>138</v>
       </c>
@@ -3682,7 +3725,7 @@
       <c r="BO30" s="35"/>
       <c r="BP30" s="34"/>
     </row>
-    <row r="31" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="29" t="s">
         <v>138</v>
       </c>
@@ -3970,7 +4013,7 @@
       <c r="BO32" s="35"/>
       <c r="BP32" s="34"/>
     </row>
-    <row r="33" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="29" t="s">
         <v>138</v>
       </c>
@@ -4114,7 +4157,7 @@
       <c r="BO33" s="35"/>
       <c r="BP33" s="34"/>
     </row>
-    <row r="34" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="29" t="s">
         <v>138</v>
       </c>
@@ -4258,7 +4301,7 @@
       <c r="BO34" s="35"/>
       <c r="BP34" s="34"/>
     </row>
-    <row r="35" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="29" t="s">
         <v>138</v>
       </c>
@@ -4402,7 +4445,7 @@
       <c r="BO35" s="35"/>
       <c r="BP35" s="34"/>
     </row>
-    <row r="36" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="29" t="s">
         <v>138</v>
       </c>
@@ -4546,7 +4589,7 @@
       <c r="BO36" s="35"/>
       <c r="BP36" s="34"/>
     </row>
-    <row r="37" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="29" t="s">
         <v>138</v>
       </c>
@@ -4690,7 +4733,7 @@
       <c r="BO37" s="35"/>
       <c r="BP37" s="34"/>
     </row>
-    <row r="38" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="29" t="s">
         <v>138</v>
       </c>
@@ -4836,7 +4879,7 @@
       <c r="BO38" s="35"/>
       <c r="BP38" s="34"/>
     </row>
-    <row r="39" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="29" t="s">
         <v>138</v>
       </c>
@@ -4980,7 +5023,7 @@
       <c r="BO39" s="35"/>
       <c r="BP39" s="34"/>
     </row>
-    <row r="40" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="29" t="s">
         <v>138</v>
       </c>
@@ -5270,7 +5313,7 @@
       <c r="BO41" s="35"/>
       <c r="BP41" s="34"/>
     </row>
-    <row r="42" spans="1:68" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:68" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="29" t="s">
         <v>138</v>
       </c>
@@ -5419,7 +5462,13 @@
       <c r="BP42" s="34"/>
     </row>
   </sheetData>
-  <autoFilter ref="A27:BP27" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A27:BP42" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="49">
+      <filters>
+        <filter val="0000159010"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="7">
     <mergeCell ref="A6:A11"/>
     <mergeCell ref="B6:B11"/>
@@ -5597,46 +5646,46 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD021527-37FD-4C54-9F30-14DD15DB7F36}">
-  <dimension ref="A2:M25"/>
+  <dimension ref="A2:O28"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.7265625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="46.7265625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="28.453125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="24.54296875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="29.81640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="26.54296875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="24.453125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="29.26953125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.54296875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="23" style="1" customWidth="1"/>
-    <col min="12" max="12" width="11.26953125" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="12.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7265625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="46.7265625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="24.54296875" style="1" customWidth="1"/>
+    <col min="6" max="7" width="12.453125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="29.81640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="26.54296875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="24.453125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="29.26953125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="26.54296875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="23" style="1" customWidth="1"/>
+    <col min="14" max="14" width="11.26953125" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="5" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="38" t="s">
+    <row r="4" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="5" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="39"/>
       <c r="C5" s="39"/>
       <c r="D5" s="39"/>
       <c r="E5" s="39"/>
@@ -5645,385 +5694,596 @@
       <c r="H5" s="39"/>
       <c r="I5" s="39"/>
       <c r="J5" s="39"/>
-      <c r="K5" s="40"/>
-    </row>
-    <row r="6" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="7" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="3" t="s">
+      <c r="K5" s="39"/>
+      <c r="L5" s="39"/>
+      <c r="M5" s="40"/>
+    </row>
+    <row r="6" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="H6" s="1" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="41" t="s">
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="42"/>
-      <c r="I7" s="43" t="s">
+      <c r="I7" s="42"/>
+      <c r="K7" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="J7" s="44"/>
-    </row>
-    <row r="8" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="5" t="s">
+      <c r="L7" s="44"/>
+    </row>
+    <row r="8" spans="1:15" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="H8" s="51"/>
+      <c r="I8" s="51"/>
+      <c r="K8" s="52"/>
+      <c r="L8" s="52"/>
+    </row>
+    <row r="9" spans="1:15" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="54" t="str">
+        <f>'CTR '!R27</f>
+        <v>Contract ID</v>
+      </c>
+      <c r="B9" s="55" t="str">
+        <f>'CTR '!AX27</f>
+        <v>Account Number</v>
+      </c>
+      <c r="C9" s="53" t="str">
+        <f>'CTR '!AY27</f>
+        <v>Account Name</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="F9" s="56" t="str">
+        <f>'CTR '!BF27</f>
+        <v>Contract Currency</v>
+      </c>
+      <c r="G9" s="56"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="51"/>
+      <c r="J9" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="K9" s="52"/>
+      <c r="L9" s="52"/>
+    </row>
+    <row r="10" spans="1:15" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="D10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="F10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="G10" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="H10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="I10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="J10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="K10" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="L10" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="M10" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="s">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A11" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="C11" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="D11" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="E11" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="F11" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="F9" s="13">
+      <c r="G11" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="H11" s="13">
         <v>-113405.22</v>
       </c>
-      <c r="G9" s="13">
+      <c r="I11" s="13">
         <v>-789300.30999999994</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="J11" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="15">
-        <f>G9</f>
+      <c r="K11" s="11"/>
+      <c r="L11" s="15">
+        <f>I11</f>
         <v>-789300.30999999994</v>
       </c>
-      <c r="K9" s="16">
-        <f t="shared" ref="K9:K14" si="0">G9-J9</f>
+      <c r="M11" s="16">
+        <f t="shared" ref="M11:M16" si="0">I11-L11</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="s">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A12" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="C12" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="D12" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="E12" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="F12" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="F10" s="13">
+      <c r="G12" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="H12" s="13">
         <v>164.94000000000233</v>
       </c>
-      <c r="G10" s="13">
+      <c r="I12" s="13">
         <v>156.77999999999884</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="J12" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I10" s="11"/>
-      <c r="J10" s="15">
-        <f>G10</f>
+      <c r="K12" s="11"/>
+      <c r="L12" s="15">
+        <f>I12</f>
         <v>156.77999999999884</v>
       </c>
-      <c r="K10" s="16">
+      <c r="M12" s="16">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A11" s="9" t="s">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A13" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="C13" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="D13" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="E13" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="F13" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="F11" s="13">
+      <c r="G13" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="H13" s="13">
         <v>-2466.4499999999998</v>
       </c>
-      <c r="G11" s="13">
+      <c r="I13" s="13">
         <v>-17083.400000000001</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="J13" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="I11" s="11">
+      <c r="K13" s="11">
         <v>6.91</v>
       </c>
-      <c r="J11" s="15">
-        <f>I11*F11</f>
+      <c r="L13" s="15">
+        <f>K13*H13</f>
         <v>-17043.1695</v>
       </c>
-      <c r="K11" s="16">
-        <f t="shared" si="0"/>
+      <c r="M13" s="16">
+        <f>I13-L13</f>
         <v>-40.230500000001484</v>
       </c>
-      <c r="M11" s="17"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="s">
+      <c r="O13" s="17"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A14" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B14" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="C14" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="D14" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="E14" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="F14" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="F12" s="13">
+      <c r="G14" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="H14" s="13">
         <v>140238.31</v>
       </c>
-      <c r="G12" s="13">
+      <c r="I14" s="13">
         <v>976058.64</v>
       </c>
-      <c r="H12" s="14" t="s">
+      <c r="J14" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I12" s="11"/>
-      <c r="J12" s="15">
-        <f>G12</f>
+      <c r="K14" s="11"/>
+      <c r="L14" s="15">
+        <f>I14</f>
         <v>976058.64</v>
       </c>
-      <c r="K12" s="16">
+      <c r="M14" s="16">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M12" s="17"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A13" s="9" t="s">
+      <c r="O14" s="17"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A15" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="C15" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="D15" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="E15" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="F15" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="F13" s="13">
+      <c r="G15" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="H15" s="13">
         <v>-29.27</v>
       </c>
-      <c r="G13" s="13">
+      <c r="I15" s="13">
         <v>-202.72</v>
       </c>
-      <c r="H13" s="14" t="s">
+      <c r="J15" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="I13" s="11">
+      <c r="K15" s="11">
         <v>6.91</v>
       </c>
-      <c r="J13" s="15">
-        <f t="shared" ref="J13:J15" si="1">I13*F13</f>
+      <c r="L15" s="15">
+        <f t="shared" ref="L15:L17" si="1">K15*H15</f>
         <v>-202.25569999999999</v>
       </c>
-      <c r="K13" s="16">
+      <c r="M15" s="16">
         <f t="shared" si="0"/>
         <v>-0.46430000000000859</v>
       </c>
-      <c r="L13" s="18"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
+      <c r="N15" s="18"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A16" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="C16" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="D16" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="E16" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="F16" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="F14" s="13">
+      <c r="G16" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="H16" s="13">
         <v>-26955.02</v>
       </c>
-      <c r="G14" s="13">
+      <c r="I16" s="13">
         <v>-186698.83</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="J16" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="I14" s="11">
+      <c r="K16" s="11">
         <v>6.91</v>
       </c>
-      <c r="J14" s="15">
+      <c r="L16" s="15">
         <f t="shared" si="1"/>
         <v>-186259.1882</v>
       </c>
-      <c r="K14" s="16">
+      <c r="M16" s="16">
         <f t="shared" si="0"/>
         <v>-439.64179999998305</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A15" s="9" t="s">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A17" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="C17" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="D17" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="E17" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="F17" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="F15" s="13">
+      <c r="G17" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="H17" s="13">
         <v>0</v>
       </c>
-      <c r="G15" s="13">
+      <c r="I17" s="13">
         <v>0</v>
       </c>
-      <c r="H15" s="14" t="s">
+      <c r="J17" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="I15" s="11">
+      <c r="K17" s="11">
         <v>6.91</v>
       </c>
-      <c r="J15" s="15">
+      <c r="L17" s="15">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K15" s="16">
-        <f>G15-J15</f>
+      <c r="M17" s="16">
+        <f>I17-L17</f>
         <v>0</v>
       </c>
-      <c r="M15" s="17"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="F16" s="19"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="21"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22">
-        <f>SUM(K9:K15)</f>
+      <c r="O17" s="17"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="H18" s="19"/>
+      <c r="I18" s="20"/>
+      <c r="J18" s="21"/>
+      <c r="L18" s="22"/>
+      <c r="M18" s="22">
+        <f>SUM(M11:M17)</f>
         <v>-480.33659999998451</v>
       </c>
     </row>
-    <row r="17" spans="6:11" x14ac:dyDescent="0.35">
-      <c r="F17" s="19"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="21"/>
-      <c r="J17" s="23" t="s">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="H19" s="19"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="21"/>
+      <c r="L19" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="K17" s="24">
+      <c r="M19" s="24">
         <v>479.86</v>
       </c>
     </row>
-    <row r="18" spans="6:11" x14ac:dyDescent="0.35">
-      <c r="F18" s="19"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="21"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="25">
-        <f>SUM(K16:K17)</f>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B20" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="H20" s="19"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="21"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="25">
+        <f>SUM(M18:M19)</f>
         <v>-0.47659999998450076</v>
       </c>
     </row>
-    <row r="19" spans="6:11" x14ac:dyDescent="0.35">
-      <c r="F19" s="19"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="21"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="22"/>
-    </row>
-    <row r="20" spans="6:11" x14ac:dyDescent="0.35">
-      <c r="F20" s="19"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="21"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
-    </row>
-    <row r="21" spans="6:11" x14ac:dyDescent="0.35">
-      <c r="F21" s="19"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="21"/>
-      <c r="J21" s="22"/>
-      <c r="K21" s="22"/>
-    </row>
-    <row r="22" spans="6:11" x14ac:dyDescent="0.35">
-      <c r="F22" s="19"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="21"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="22"/>
-    </row>
-    <row r="24" spans="6:11" x14ac:dyDescent="0.35">
-      <c r="I24" s="22"/>
-    </row>
-    <row r="25" spans="6:11" x14ac:dyDescent="0.35">
-      <c r="I25" s="22"/>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" s="19"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="21"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="22"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B22" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="H22" s="19"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="21"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="22"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B23" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="H23" s="19"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="21"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="22"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B24" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="H24" s="19"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="21"/>
+      <c r="L24" s="22"/>
+      <c r="M24" s="22"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B25" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B26" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="K26" s="22"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B27" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="K27" s="22"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B28" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>31</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="B5:M5"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="K7:L7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>